<commit_message>
Add vision sense demo and primitives
Introduce a vision-sense feature and related primitives: add demos/uielement_vision_sense.py (NiceGUI demo and VisionSenseCodec that converts a 32-bit TIFF to a filtered PNG data URI), add game/primitives/senses.py (Sense, SenseType, Sensor/Emitter scaffolding and XLSX-backed tables), and include the vision_chart.tif asset and a small gui.forms.sense placeholder. Update main.py to run the new demo on startup and relax .gitignore to ignore image source files but keep vision_chart.tif tracked. Minor edits: add a descriptive header docstring to sophont/attributes/base.py and add sophont/attributes/body.py with basic body/brain datatypes. Also update the binary T5Mappings.xlsx file.
</commit_message>
<xml_diff>
--- a/game/primitives/T5Mappings.xlsx
+++ b/game/primitives/T5Mappings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Python\Sophont\game\mappings\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Python\Sophont\game\primitives\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5B655BFD-50A7-4744-9B3D-CC77497C4089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3ED0BBDD-B1FA-4C6F-8CEC-784BD5D2D28C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7500" yWindow="1380" windowWidth="16020" windowHeight="18180" firstSheet="1" activeTab="2" xr2:uid="{922B48FF-0A11-4648-9808-3CC4D7F2A9F4}"/>
+    <workbookView xWindow="10875" yWindow="1680" windowWidth="22995" windowHeight="18510" firstSheet="11" activeTab="11" xr2:uid="{922B48FF-0A11-4648-9808-3CC4D7F2A9F4}"/>
   </bookViews>
   <sheets>
     <sheet name="characteristics.master.en" sheetId="9" r:id="rId1"/>
@@ -24,8 +24,14 @@
     <sheet name="knowledges.base.en" sheetId="6" r:id="rId9"/>
     <sheet name="knowledges.skills.form" sheetId="7" r:id="rId10"/>
     <sheet name="knowledges.skills.data" sheetId="8" r:id="rId11"/>
+    <sheet name="vision.senses.en" sheetId="15" r:id="rId12"/>
+    <sheet name="hearing.senses.en" sheetId="16" r:id="rId13"/>
+    <sheet name="smell.senses.en" sheetId="17" r:id="rId14"/>
+    <sheet name="touch.senses.en" sheetId="18" r:id="rId15"/>
+    <sheet name="perception.senses.en" sheetId="19" r:id="rId16"/>
+    <sheet name="awareness.senses.en" sheetId="20" r:id="rId17"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -68,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="701" uniqueCount="384">
   <si>
     <t>Code</t>
   </si>
@@ -770,6 +776,456 @@
   </si>
   <si>
     <t>engineering</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Wavelength</t>
+  </si>
+  <si>
+    <t>Star</t>
+  </si>
+  <si>
+    <t>Extended Color Name</t>
+  </si>
+  <si>
+    <t>v</t>
+  </si>
+  <si>
+    <t>h</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>u</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>r</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>n</t>
+  </si>
+  <si>
+    <t>i</t>
+  </si>
+  <si>
+    <t>f</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>z</t>
+  </si>
+  <si>
+    <t>vharduv</t>
+  </si>
+  <si>
+    <t>harduv</t>
+  </si>
+  <si>
+    <t>darkuv</t>
+  </si>
+  <si>
+    <t>uv</t>
+  </si>
+  <si>
+    <t>sparkle</t>
+  </si>
+  <si>
+    <t>purple</t>
+  </si>
+  <si>
+    <t>blue</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>cerise</t>
+  </si>
+  <si>
+    <t>aglow</t>
+  </si>
+  <si>
+    <t>nearir</t>
+  </si>
+  <si>
+    <t>ir</t>
+  </si>
+  <si>
+    <t>farir</t>
+  </si>
+  <si>
+    <t>xir</t>
+  </si>
+  <si>
+    <t>zir</t>
+  </si>
+  <si>
+    <t>B0 I</t>
+  </si>
+  <si>
+    <t>B0 V</t>
+  </si>
+  <si>
+    <t>B5 V</t>
+  </si>
+  <si>
+    <t>B9 V</t>
+  </si>
+  <si>
+    <t>A2 V</t>
+  </si>
+  <si>
+    <t>A9 V</t>
+  </si>
+  <si>
+    <t>F7 V</t>
+  </si>
+  <si>
+    <t>G2 V</t>
+  </si>
+  <si>
+    <t>K1 V</t>
+  </si>
+  <si>
+    <t>K4 V</t>
+  </si>
+  <si>
+    <t>K7 V</t>
+  </si>
+  <si>
+    <t>M0 V</t>
+  </si>
+  <si>
+    <t>M2 V</t>
+  </si>
+  <si>
+    <t>M5 V</t>
+  </si>
+  <si>
+    <t>L9 VI</t>
+  </si>
+  <si>
+    <t>T7 VI</t>
+  </si>
+  <si>
+    <t>human visible green</t>
+  </si>
+  <si>
+    <t>human visible red</t>
+  </si>
+  <si>
+    <t>human visible cerise</t>
+  </si>
+  <si>
+    <t>very hard ultra violet</t>
+  </si>
+  <si>
+    <t>hard ultra violet</t>
+  </si>
+  <si>
+    <t>dark ultra violet</t>
+  </si>
+  <si>
+    <t>ultra violet</t>
+  </si>
+  <si>
+    <t>near ultra violet</t>
+  </si>
+  <si>
+    <t>human visible violet</t>
+  </si>
+  <si>
+    <t>human visible blue</t>
+  </si>
+  <si>
+    <t>edge of infrared</t>
+  </si>
+  <si>
+    <t>near infra red</t>
+  </si>
+  <si>
+    <t>infra red</t>
+  </si>
+  <si>
+    <t>far infra red</t>
+  </si>
+  <si>
+    <t>extreme infra red</t>
+  </si>
+  <si>
+    <t>beyond extreme ir</t>
+  </si>
+  <si>
+    <t>Frequency</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>delta</t>
+  </si>
+  <si>
+    <t>theta</t>
+  </si>
+  <si>
+    <t>alpha</t>
+  </si>
+  <si>
+    <t>beta</t>
+  </si>
+  <si>
+    <t>gamma</t>
+  </si>
+  <si>
+    <t>middle c</t>
+  </si>
+  <si>
+    <t>dog whistle</t>
+  </si>
+  <si>
+    <t>bats</t>
+  </si>
+  <si>
+    <t>Pheromone</t>
+  </si>
+  <si>
+    <t>Intensity</t>
+  </si>
+  <si>
+    <t>Odourless</t>
+  </si>
+  <si>
+    <t>Slight</t>
+  </si>
+  <si>
+    <t>Aromatic</t>
+  </si>
+  <si>
+    <t>Strong</t>
+  </si>
+  <si>
+    <t>Intense</t>
+  </si>
+  <si>
+    <t>Overwhelming</t>
+  </si>
+  <si>
+    <t>Trail Marker</t>
+  </si>
+  <si>
+    <t>Alarm</t>
+  </si>
+  <si>
+    <t>Gender Attractor</t>
+  </si>
+  <si>
+    <t>Fear</t>
+  </si>
+  <si>
+    <t>Repellent</t>
+  </si>
+  <si>
+    <t>Gender Balancer</t>
+  </si>
+  <si>
+    <t>Mood Soother</t>
+  </si>
+  <si>
+    <t>Caste Balancer</t>
+  </si>
+  <si>
+    <t>Caste Determiner</t>
+  </si>
+  <si>
+    <t>Gender Change Trigger</t>
+  </si>
+  <si>
+    <t>Caste Change Trigger</t>
+  </si>
+  <si>
+    <t>Sense Damper</t>
+  </si>
+  <si>
+    <t>Sense Enhancer</t>
+  </si>
+  <si>
+    <t>Royalty Marker</t>
+  </si>
+  <si>
+    <t>Universal Compeller</t>
+  </si>
+  <si>
+    <t>Dread</t>
+  </si>
+  <si>
+    <t>Courage</t>
+  </si>
+  <si>
+    <t>Shun</t>
+  </si>
+  <si>
+    <t>Berserk</t>
+  </si>
+  <si>
+    <t>Scatter</t>
+  </si>
+  <si>
+    <t>Unknown</t>
+  </si>
+  <si>
+    <t>Special</t>
+  </si>
+  <si>
+    <t>Ultimate</t>
+  </si>
+  <si>
+    <t>Descriptor</t>
+  </si>
+  <si>
+    <t>Smooth</t>
+  </si>
+  <si>
+    <t>Xfaint</t>
+  </si>
+  <si>
+    <t>Faint</t>
+  </si>
+  <si>
+    <t>VFaint</t>
+  </si>
+  <si>
+    <t>VSmall</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Grooved</t>
+  </si>
+  <si>
+    <t>Coarse</t>
+  </si>
+  <si>
+    <t>Rough</t>
+  </si>
+  <si>
+    <t>VRough</t>
+  </si>
+  <si>
+    <t>XRough</t>
+  </si>
+  <si>
+    <t>DiceNum</t>
+  </si>
+  <si>
+    <t>Tone</t>
+  </si>
+  <si>
+    <t>Poice</t>
+  </si>
+  <si>
+    <t>dominating</t>
+  </si>
+  <si>
+    <t>very intelligent</t>
+  </si>
+  <si>
+    <t>intelligent</t>
+  </si>
+  <si>
+    <t>sapient</t>
+  </si>
+  <si>
+    <t>concious</t>
+  </si>
+  <si>
+    <t>rudimentary</t>
+  </si>
+  <si>
+    <t>artificial</t>
+  </si>
+  <si>
+    <t>stange</t>
+  </si>
+  <si>
+    <t>bizarre</t>
+  </si>
+  <si>
+    <t>whine</t>
+  </si>
+  <si>
+    <t>faint</t>
+  </si>
+  <si>
+    <t>vague</t>
+  </si>
+  <si>
+    <t>common</t>
+  </si>
+  <si>
+    <t>firm</t>
+  </si>
+  <si>
+    <t>strong</t>
+  </si>
+  <si>
+    <t>powerful</t>
+  </si>
+  <si>
+    <t>blast</t>
+  </si>
+  <si>
+    <t>overwhelming</t>
+  </si>
+  <si>
+    <t>Range</t>
+  </si>
+  <si>
+    <t>Mass</t>
+  </si>
+  <si>
+    <t>Electric</t>
+  </si>
+  <si>
+    <t>Magnetic</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>T</t>
   </si>
 </sst>
 </file>
@@ -3266,6 +3722,1350 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E51E3B8-5D93-48EC-9DC5-2357134CDEC1}">
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>234</v>
+      </c>
+      <c r="D1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E1" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>30</v>
+      </c>
+      <c r="B2" t="s">
+        <v>238</v>
+      </c>
+      <c r="C2" t="s">
+        <v>254</v>
+      </c>
+      <c r="D2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E2" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>100</v>
+      </c>
+      <c r="B3" t="s">
+        <v>239</v>
+      </c>
+      <c r="C3" t="s">
+        <v>255</v>
+      </c>
+      <c r="D3" t="s">
+        <v>271</v>
+      </c>
+      <c r="E3" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>170</v>
+      </c>
+      <c r="B4" t="s">
+        <v>240</v>
+      </c>
+      <c r="C4" t="s">
+        <v>256</v>
+      </c>
+      <c r="D4" t="s">
+        <v>272</v>
+      </c>
+      <c r="E4" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>240</v>
+      </c>
+      <c r="B5" t="s">
+        <v>241</v>
+      </c>
+      <c r="C5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D5" t="s">
+        <v>273</v>
+      </c>
+      <c r="E5" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>310</v>
+      </c>
+      <c r="B6" t="s">
+        <v>242</v>
+      </c>
+      <c r="C6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D6" t="s">
+        <v>274</v>
+      </c>
+      <c r="E6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>380</v>
+      </c>
+      <c r="B7" t="s">
+        <v>243</v>
+      </c>
+      <c r="C7" t="s">
+        <v>259</v>
+      </c>
+      <c r="D7" t="s">
+        <v>275</v>
+      </c>
+      <c r="E7" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>450</v>
+      </c>
+      <c r="B8" t="s">
+        <v>244</v>
+      </c>
+      <c r="C8" t="s">
+        <v>260</v>
+      </c>
+      <c r="D8" t="s">
+        <v>276</v>
+      </c>
+      <c r="E8" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>540</v>
+      </c>
+      <c r="B9" t="s">
+        <v>245</v>
+      </c>
+      <c r="C9" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" t="s">
+        <v>277</v>
+      </c>
+      <c r="E9" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>610</v>
+      </c>
+      <c r="B10" t="s">
+        <v>246</v>
+      </c>
+      <c r="C10" t="s">
+        <v>262</v>
+      </c>
+      <c r="D10" t="s">
+        <v>278</v>
+      </c>
+      <c r="E10" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>680</v>
+      </c>
+      <c r="B11" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" t="s">
+        <v>263</v>
+      </c>
+      <c r="D11" t="s">
+        <v>279</v>
+      </c>
+      <c r="E11" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>750</v>
+      </c>
+      <c r="B12" t="s">
+        <v>248</v>
+      </c>
+      <c r="C12" t="s">
+        <v>264</v>
+      </c>
+      <c r="D12" t="s">
+        <v>280</v>
+      </c>
+      <c r="E12" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>820</v>
+      </c>
+      <c r="B13" t="s">
+        <v>249</v>
+      </c>
+      <c r="C13" t="s">
+        <v>265</v>
+      </c>
+      <c r="D13" t="s">
+        <v>281</v>
+      </c>
+      <c r="E13" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>890</v>
+      </c>
+      <c r="B14" t="s">
+        <v>250</v>
+      </c>
+      <c r="C14" t="s">
+        <v>266</v>
+      </c>
+      <c r="D14" t="s">
+        <v>282</v>
+      </c>
+      <c r="E14" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>1000</v>
+      </c>
+      <c r="B15" t="s">
+        <v>251</v>
+      </c>
+      <c r="C15" t="s">
+        <v>267</v>
+      </c>
+      <c r="D15" t="s">
+        <v>283</v>
+      </c>
+      <c r="E15" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>2000</v>
+      </c>
+      <c r="B16" t="s">
+        <v>252</v>
+      </c>
+      <c r="C16" t="s">
+        <v>268</v>
+      </c>
+      <c r="D16" t="s">
+        <v>284</v>
+      </c>
+      <c r="E16" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>4000</v>
+      </c>
+      <c r="B17" t="s">
+        <v>253</v>
+      </c>
+      <c r="C17" t="s">
+        <v>269</v>
+      </c>
+      <c r="D17" t="s">
+        <v>285</v>
+      </c>
+      <c r="E17" t="s">
+        <v>301</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2928D82E-606D-41E3-BC28-08DC9E77311B}">
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="10" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>302</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>303</v>
+      </c>
+      <c r="D1" t="s">
+        <v>304</v>
+      </c>
+      <c r="E1" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2">
+        <v>-3</v>
+      </c>
+      <c r="E2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>4</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3">
+        <v>-2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>8</v>
+      </c>
+      <c r="B4">
+        <v>3</v>
+      </c>
+      <c r="C4">
+        <v>3</v>
+      </c>
+      <c r="D4">
+        <v>-1</v>
+      </c>
+      <c r="E4" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>16</v>
+      </c>
+      <c r="B5">
+        <v>4</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>32</v>
+      </c>
+      <c r="B6">
+        <v>5</v>
+      </c>
+      <c r="C6">
+        <v>5</v>
+      </c>
+      <c r="D6">
+        <v>1</v>
+      </c>
+      <c r="E6" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>64</v>
+      </c>
+      <c r="B7">
+        <v>6</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
+      </c>
+      <c r="D7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>128</v>
+      </c>
+      <c r="B8">
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <v>7</v>
+      </c>
+      <c r="D8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>256</v>
+      </c>
+      <c r="B9">
+        <v>8</v>
+      </c>
+      <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>4</v>
+      </c>
+      <c r="E9" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>512</v>
+      </c>
+      <c r="B10">
+        <v>9</v>
+      </c>
+      <c r="C10">
+        <v>9</v>
+      </c>
+      <c r="D10">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>1000</v>
+      </c>
+      <c r="B11">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <v>10</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2000</v>
+      </c>
+      <c r="B12">
+        <v>11</v>
+      </c>
+      <c r="C12">
+        <v>11</v>
+      </c>
+      <c r="D12">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>4000</v>
+      </c>
+      <c r="B13">
+        <v>12</v>
+      </c>
+      <c r="C13">
+        <v>12</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>8000</v>
+      </c>
+      <c r="B14">
+        <v>13</v>
+      </c>
+      <c r="C14">
+        <v>13</v>
+      </c>
+      <c r="D14">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>16000</v>
+      </c>
+      <c r="B15">
+        <v>14</v>
+      </c>
+      <c r="C15">
+        <v>14</v>
+      </c>
+      <c r="D15">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>32000</v>
+      </c>
+      <c r="B16">
+        <v>15</v>
+      </c>
+      <c r="C16">
+        <v>15</v>
+      </c>
+      <c r="D16">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>64000</v>
+      </c>
+      <c r="B17">
+        <v>16</v>
+      </c>
+      <c r="C17">
+        <v>16</v>
+      </c>
+      <c r="D17">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>128000</v>
+      </c>
+      <c r="B18">
+        <v>17</v>
+      </c>
+      <c r="C18">
+        <v>17</v>
+      </c>
+      <c r="D18">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>256000</v>
+      </c>
+      <c r="B19">
+        <v>18</v>
+      </c>
+      <c r="C19">
+        <v>18</v>
+      </c>
+      <c r="D19">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>524288</v>
+      </c>
+      <c r="B20">
+        <v>19</v>
+      </c>
+      <c r="C20">
+        <v>19</v>
+      </c>
+      <c r="D20">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59B464F1-0237-4218-A99B-FF20C756E199}">
+  <dimension ref="A1:C35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="8.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>314</v>
+      </c>
+      <c r="C1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>344</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5A879DF-5176-4F8C-B235-7B10484AB2C8}">
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>-5</v>
+      </c>
+      <c r="B2" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>-4</v>
+      </c>
+      <c r="B3" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>-3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>-2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>-1</v>
+      </c>
+      <c r="B6" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>0</v>
+      </c>
+      <c r="B7" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>2</v>
+      </c>
+      <c r="B9" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>3</v>
+      </c>
+      <c r="B10" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>4</v>
+      </c>
+      <c r="B11" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>5</v>
+      </c>
+      <c r="B12" t="s">
+        <v>356</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A398146-A5F4-4D8B-9FAB-B0FE0C6CA455}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>357</v>
+      </c>
+      <c r="C1" t="s">
+        <v>358</v>
+      </c>
+      <c r="D1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>360</v>
+      </c>
+      <c r="D2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>361</v>
+      </c>
+      <c r="D3" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>362</v>
+      </c>
+      <c r="D4" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>363</v>
+      </c>
+      <c r="D5" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>364</v>
+      </c>
+      <c r="D6" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>365</v>
+      </c>
+      <c r="D7" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>6</v>
+      </c>
+      <c r="C8" t="s">
+        <v>366</v>
+      </c>
+      <c r="D8" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>7</v>
+      </c>
+      <c r="C9" t="s">
+        <v>367</v>
+      </c>
+      <c r="D9" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>368</v>
+      </c>
+      <c r="D10" t="s">
+        <v>377</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A81A712D-FBBA-4486-9172-7EC97A2BE659}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>378</v>
+      </c>
+      <c r="C1" t="s">
+        <v>379</v>
+      </c>
+      <c r="D1" t="s">
+        <v>380</v>
+      </c>
+      <c r="E1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>0</v>
+      </c>
+      <c r="B2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>382</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>383</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>3</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>4</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>5</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+      <c r="C7">
+        <v>5</v>
+      </c>
+      <c r="D7">
+        <v>3</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>6</v>
+      </c>
+      <c r="B8">
+        <v>4</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8">
+        <v>4</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>5</v>
+      </c>
+      <c r="C9">
+        <v>7</v>
+      </c>
+      <c r="D9">
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>6</v>
+      </c>
+      <c r="C10">
+        <v>8</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+      <c r="E10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>7</v>
+      </c>
+      <c r="C11">
+        <v>9</v>
+      </c>
+      <c r="D11">
+        <v>7</v>
+      </c>
+      <c r="E11">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6EA884A-79BB-4D85-BC1A-03A86D7E0947}">
   <sheetPr>

</xml_diff>